<commit_message>
fix: enforce all required transport modes
</commit_message>
<xml_diff>
--- a/site/public/beego-engineers-template.xlsx
+++ b/site/public/beego-engineers-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инженеры" sheetId="1" r:id="R3a9ec1751cb74874"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пояснения" sheetId="2" r:id="R20bf256275a74d2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инженеры" sheetId="1" r:id="R7dcbdf06e94a4aee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пояснения" sheetId="2" r:id="R21db4ebef8914daa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8537,7 +8537,7 @@
   </x:sheetData>
   <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="F2:F5000">
-      <x:formula1>"CAR,PUBLIC_TRANSIT,FOOT,BIKE"</x:formula1>
+      <x:formula1>"CAR,PUBLIC_TRANSIT,WALKING,BICYCLE"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L2:L5000">
       <x:formula1>"AVAILABLE,UNAVAILABLE"</x:formula1>
@@ -8666,7 +8666,7 @@
         <x:v>Тип транспорта</x:v>
       </x:c>
       <x:c r="D8" s="27" t="str">
-        <x:v>CAR / PUBLIC_TRANSIT / FOOT / BIKE</x:v>
+        <x:v>CAR / PUBLIC_TRANSIT / WALKING / BICYCLE</x:v>
       </x:c>
       <x:c r="E8" s="27" t="str">
         <x:v>CAR</x:v>

</xml_diff>